<commit_message>
Taxonomy review decisions: microsporidia in Fungi, accepted names, missing protozoa
- all microsporidia in the Fungi (1,394 names of v3.0.1 from P_ to F_, old codes translated by name)
- Enterocytozoon bieneusi and Encephalitozoon cuniculi as accepted names (accepted_name_override)
- Balantidium and Isospora added to MO_RELEVANT_GENERA; Cystoisospora belli as synonym of Isospora belli
- synonym cycles decided: Capillidium and Scolecobasidium are the current genera
- removed the stale data-raw/taxonomy_lpsn0.rds
- microorganisms now has 107,253 records; all tests pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/datasets/microorganisms.codes.xlsx
+++ b/data-raw/datasets/microorganisms.codes.xlsx
@@ -4974,7 +4974,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>P_NCLSP_SLMN</t>
+          <t>F_NCLSPR_SLMN</t>
         </is>
       </c>
     </row>
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B2359" t="inlineStr">
         <is>
-          <t>P_ENCPH_BINS</t>
+          <t>F_ENCPH_BINS</t>
         </is>
       </c>
     </row>
@@ -29946,7 +29946,7 @@
       </c>
       <c r="B2465" t="inlineStr">
         <is>
-          <t>P_ENCPH</t>
+          <t>F_ENCPH</t>
         </is>
       </c>
     </row>
@@ -30858,7 +30858,7 @@
       </c>
       <c r="B2541" t="inlineStr">
         <is>
-          <t>P_EYTZN</t>
+          <t>F_EYTZN</t>
         </is>
       </c>
     </row>
@@ -49386,7 +49386,7 @@
       </c>
       <c r="B4085" t="inlineStr">
         <is>
-          <t>P_NOSEM</t>
+          <t>F_NOSEM</t>
         </is>
       </c>
     </row>
@@ -53562,7 +53562,7 @@
       </c>
       <c r="B4433" t="inlineStr">
         <is>
-          <t>P_PLSTP</t>
+          <t>F_PLSTP</t>
         </is>
       </c>
     </row>
@@ -61806,7 +61806,7 @@
       </c>
       <c r="B5120" t="inlineStr">
         <is>
-          <t>P_ENCPH</t>
+          <t>F_ENCPH</t>
         </is>
       </c>
     </row>
@@ -62862,7 +62862,7 @@
       </c>
       <c r="B5208" t="inlineStr">
         <is>
-          <t>P_ENCPH_INTS</t>
+          <t>F_ENCPH_INTS</t>
         </is>
       </c>
     </row>

</xml_diff>